<commit_message>
provo a togliere il wrapper
</commit_message>
<xml_diff>
--- a/export_dati/04_Step4B_Risultati_TensorFlow.xlsx
+++ b/export_dati/04_Step4B_Risultati_TensorFlow.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,36 +456,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>(50,)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D2" t="n">
         <v>0.0001</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>98.71%</t>
+          <t>98.88%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.0425201877951622</v>
+        <v>0.04074851050972939</v>
       </c>
       <c r="G2" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>(50, 25)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -494,21 +494,891 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D3" t="n">
         <v>0.0001</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>98.78%</t>
+          <t>98.91%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.04653596878051758</v>
+        <v>0.04138786718249321</v>
       </c>
       <c r="G3" t="n">
-        <v>16</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>(32,)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>98.89%</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0.04145969450473785</v>
+      </c>
+      <c r="G4" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>(32,)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>98.88%</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0.04153100028634071</v>
+      </c>
+      <c r="G5" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>(64,)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>98.91%</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0.04153378307819366</v>
+      </c>
+      <c r="G6" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>(64,)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>98.80%</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0.04193461313843727</v>
+      </c>
+      <c r="G7" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>(32,)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>98.87%</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0.04210275039076805</v>
+      </c>
+      <c r="G8" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>(64,)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>98.77%</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0.04255594313144684</v>
+      </c>
+      <c r="G9" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>(32, 16)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>98.86%</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0.04291569069027901</v>
+      </c>
+      <c r="G10" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>(32,)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>98.92%</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0.04337989911437035</v>
+      </c>
+      <c r="G11" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>(64, 32)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>98.84%</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>0.04366312548518181</v>
+      </c>
+      <c r="G12" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>(64,)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>98.82%</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>0.04399563744664192</v>
+      </c>
+      <c r="G13" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>(32,)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>98.88%</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>0.04427820816636086</v>
+      </c>
+      <c r="G14" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>(64,)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>98.86%</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0.04471180960536003</v>
+      </c>
+      <c r="G15" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>(64, 32)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>98.86%</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0.04477332532405853</v>
+      </c>
+      <c r="G16" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>(32, 16)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>98.82%</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0.04477648064494133</v>
+      </c>
+      <c r="G17" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>(64, 32)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>98.87%</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.04478396475315094</v>
+      </c>
+      <c r="G18" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>(32, 16)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>98.77%</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0.04492866992950439</v>
+      </c>
+      <c r="G19" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>(64, 32)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>98.80%</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.04536068812012672</v>
+      </c>
+      <c r="G20" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>(32,)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>98.84%</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0.0455637164413929</v>
+      </c>
+      <c r="G21" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>(32, 16)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>98.75%</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.0457637794315815</v>
+      </c>
+      <c r="G22" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>(32,)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>98.79%</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0.0462014451622963</v>
+      </c>
+      <c r="G23" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>(64,)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>98.76%</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0.04808444157242775</v>
+      </c>
+      <c r="G24" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>(64,)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>98.76%</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0.04954849556088448</v>
+      </c>
+      <c r="G25" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>(32, 16)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>98.88%</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0.05152564495801926</v>
+      </c>
+      <c r="G26" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>(32, 16)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>98.80%</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0.05457977950572968</v>
+      </c>
+      <c r="G27" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>(32, 16)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>98.93%</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0.05536512657999992</v>
+      </c>
+      <c r="G28" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>(32, 16)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>98.75%</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0.05593835189938545</v>
+      </c>
+      <c r="G29" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>(64, 32)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>98.90%</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0.05644501000642776</v>
+      </c>
+      <c r="G30" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>(64, 32)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>relu</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>98.90%</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0.05702962726354599</v>
+      </c>
+      <c r="G31" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>(64, 32)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>98.79%</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0.05944292619824409</v>
+      </c>
+      <c r="G32" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>(64, 32)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>tanh</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>98.63%</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>0.06703592836856842</v>
+      </c>
+      <c r="G33" t="n">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finito il test della rete con i risultai della TensorFLow coerenti
</commit_message>
<xml_diff>
--- a/export_dati/04_Step4B_Risultati_TensorFlow.xlsx
+++ b/export_dati/04_Step4B_Risultati_TensorFlow.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -472,25 +472,25 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>98.88%</t>
+          <t>99.02%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.04074851050972939</v>
+        <v>0.04205260798335075</v>
       </c>
       <c r="G2" t="n">
-        <v>20</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -501,20 +501,20 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>98.91%</t>
+          <t>99.00%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.04138786718249321</v>
+        <v>0.04149504005908966</v>
       </c>
       <c r="G3" t="n">
-        <v>15</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -523,27 +523,27 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D4" t="n">
         <v>0.0001</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>98.89%</t>
+          <t>98.97%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.04145969450473785</v>
+        <v>0.04121869802474976</v>
       </c>
       <c r="G4" t="n">
-        <v>13</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -559,20 +559,20 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>98.88%</t>
+          <t>98.97%</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.04153100028634071</v>
+        <v>0.04182364791631699</v>
       </c>
       <c r="G5" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -581,21 +581,21 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D6" t="n">
         <v>0.0001</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>98.91%</t>
+          <t>98.95%</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.04153378307819366</v>
+        <v>0.04152262955904007</v>
       </c>
       <c r="G6" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -613,47 +613,47 @@
         <v>0.01</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>98.80%</t>
+          <t>98.93%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.04193461313843727</v>
+        <v>0.04521772637963295</v>
       </c>
       <c r="G7" t="n">
-        <v>15</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D8" t="n">
         <v>0.0001</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>98.87%</t>
+          <t>98.92%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.04210275039076805</v>
+        <v>0.04350379481911659</v>
       </c>
       <c r="G8" t="n">
-        <v>11</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9">
@@ -671,18 +671,18 @@
         <v>0.01</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>98.77%</t>
+          <t>98.92%</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.04255594313144684</v>
+        <v>0.04663772508502007</v>
       </c>
       <c r="G9" t="n">
-        <v>9</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10">
@@ -693,25 +693,25 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>0.005</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>98.86%</t>
+          <t>98.92%</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.04291569069027901</v>
+        <v>0.05845890939235687</v>
       </c>
       <c r="G10" t="n">
-        <v>86</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11">
@@ -733,11 +733,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>98.92%</t>
+          <t>98.90%</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.04337989911437035</v>
+        <v>0.04516733437776566</v>
       </c>
       <c r="G11" t="n">
         <v>200</v>
@@ -746,59 +746,59 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D12" t="n">
         <v>0.0001</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>98.84%</t>
+          <t>98.90%</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.04366312548518181</v>
+        <v>0.04540383443236351</v>
       </c>
       <c r="G12" t="n">
-        <v>49</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>0.005</v>
       </c>
       <c r="D13" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>98.82%</t>
+          <t>98.88%</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.04399563744664192</v>
+        <v>0.04486606270074844</v>
       </c>
       <c r="G13" t="n">
-        <v>200</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14">
@@ -824,50 +824,50 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.04427820816636086</v>
+        <v>0.0464915819466114</v>
       </c>
       <c r="G14" t="n">
-        <v>166</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>98.86%</t>
+          <t>98.88%</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.04471180960536003</v>
+        <v>0.04793679341673851</v>
       </c>
       <c r="G15" t="n">
-        <v>123</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -878,20 +878,20 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>98.86%</t>
+          <t>98.87%</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.04477332532405853</v>
+        <v>0.04220666736364365</v>
       </c>
       <c r="G16" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -900,79 +900,79 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>98.82%</t>
+          <t>98.85%</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.04477648064494133</v>
+        <v>0.04605346545577049</v>
       </c>
       <c r="G17" t="n">
-        <v>47</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>0.005</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>98.87%</t>
+          <t>98.85%</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.04478396475315094</v>
+        <v>0.04706387966871262</v>
       </c>
       <c r="G18" t="n">
-        <v>37</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>98.77%</t>
+          <t>98.85%</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.04492866992950439</v>
+        <v>0.04848089441657066</v>
       </c>
       <c r="G19" t="n">
-        <v>29</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20">
@@ -994,20 +994,20 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>98.80%</t>
+          <t>98.83%</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.04536068812012672</v>
+        <v>0.04578438401222229</v>
       </c>
       <c r="G20" t="n">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1016,27 +1016,27 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D21" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>98.84%</t>
+          <t>98.83%</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.0455637164413929</v>
+        <v>0.04697543010115623</v>
       </c>
       <c r="G21" t="n">
-        <v>108</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1045,21 +1045,21 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>98.75%</t>
+          <t>98.83%</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.0457637794315815</v>
+        <v>0.05896245688199997</v>
       </c>
       <c r="G22" t="n">
-        <v>20</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23">
@@ -1081,11 +1081,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>98.79%</t>
+          <t>98.82%</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.0462014451622963</v>
+        <v>0.04553953930735588</v>
       </c>
       <c r="G23" t="n">
         <v>200</v>
@@ -1094,7 +1094,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1103,56 +1103,56 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D24" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>98.76%</t>
+          <t>98.80%</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.04808444157242775</v>
+        <v>0.04541318118572235</v>
       </c>
       <c r="G24" t="n">
-        <v>136</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D25" t="n">
         <v>0.01</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>98.76%</t>
+          <t>98.80%</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.04954849556088448</v>
+        <v>0.06689533591270447</v>
       </c>
       <c r="G25" t="n">
-        <v>51</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1164,24 +1164,24 @@
         <v>0.01</v>
       </c>
       <c r="D26" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>98.88%</t>
+          <t>98.78%</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.05152564495801926</v>
+        <v>0.04281177371740341</v>
       </c>
       <c r="G26" t="n">
-        <v>200</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1190,32 +1190,32 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D27" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>98.80%</t>
+          <t>98.78%</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.05457977950572968</v>
+        <v>0.0431537926197052</v>
       </c>
       <c r="G27" t="n">
-        <v>200</v>
+        <v>28</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1226,14 +1226,14 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>98.93%</t>
+          <t>98.77%</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.05536512657999992</v>
+        <v>0.05993777886033058</v>
       </c>
       <c r="G28" t="n">
-        <v>200</v>
+        <v>154</v>
       </c>
     </row>
     <row r="29">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1259,68 +1259,68 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.05593835189938545</v>
+        <v>0.06043698638677597</v>
       </c>
       <c r="G29" t="n">
-        <v>107</v>
+        <v>200</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C30" t="n">
         <v>0.01</v>
       </c>
       <c r="D30" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>98.90%</t>
+          <t>98.73%</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.05644501000642776</v>
+        <v>0.04606348276138306</v>
       </c>
       <c r="G30" t="n">
-        <v>107</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D31" t="n">
         <v>0.01</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>98.90%</t>
+          <t>98.68%</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.05702962726354599</v>
+        <v>0.06027081981301308</v>
       </c>
       <c r="G31" t="n">
-        <v>116</v>
+        <v>198</v>
       </c>
     </row>
     <row r="32">
@@ -1331,25 +1331,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D32" t="n">
         <v>0.01</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>98.79%</t>
+          <t>98.58%</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0.05944292619824409</v>
+        <v>0.08604622632265091</v>
       </c>
       <c r="G32" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33">
@@ -1371,14 +1371,14 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>98.63%</t>
+          <t>98.30%</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0.06703592836856842</v>
+        <v>0.07404597103595734</v>
       </c>
       <c r="G33" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fino a step 1
Sistemato i commenti fino a step 1
</commit_message>
<xml_diff>
--- a/export_dati/04_Step4B_Risultati_TensorFlow.xlsx
+++ b/export_dati/04_Step4B_Risultati_TensorFlow.xlsx
@@ -465,56 +465,56 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D2" t="n">
         <v>0.0001</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>98.98%</t>
+          <t>99.45%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.04155315831303596</v>
+        <v>0.0222802422940731</v>
       </c>
       <c r="G2" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D3" t="n">
         <v>0.0001</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>98.98%</t>
+          <t>99.45%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.04191243276000023</v>
+        <v>0.0223421435803175</v>
       </c>
       <c r="G3" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -530,20 +530,20 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>98.97%</t>
+          <t>99.45%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.04121951386332512</v>
+        <v>0.02356160245835781</v>
       </c>
       <c r="G4" t="n">
-        <v>37</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -559,20 +559,20 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>98.97%</t>
+          <t>99.45%</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.04151733219623566</v>
+        <v>0.02463765628635883</v>
       </c>
       <c r="G5" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -588,43 +588,43 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>98.97%</t>
+          <t>99.43%</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.04186432808637619</v>
+        <v>0.0230771079659462</v>
       </c>
       <c r="G6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D7" t="n">
         <v>0.0001</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>98.95%</t>
+          <t>99.43%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.04161980375647545</v>
+        <v>0.02559859491884708</v>
       </c>
       <c r="G7" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8">
@@ -635,31 +635,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>98.95%</t>
+          <t>99.42%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.04558555036783218</v>
+        <v>0.02207266725599766</v>
       </c>
       <c r="G8" t="n">
-        <v>90</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -675,25 +675,25 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>98.92%</t>
+          <t>99.42%</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.04342279583215714</v>
+        <v>0.02410629577934742</v>
       </c>
       <c r="G9" t="n">
-        <v>106</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -704,25 +704,25 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>98.92%</t>
+          <t>99.42%</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.0461886040866375</v>
+        <v>0.0244292039424181</v>
       </c>
       <c r="G10" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -733,14 +733,14 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>98.92%</t>
+          <t>99.42%</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.05169887840747833</v>
+        <v>0.0225406214594841</v>
       </c>
       <c r="G11" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -758,116 +758,116 @@
         <v>0.005</v>
       </c>
       <c r="D12" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>98.90%</t>
+          <t>99.42%</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.04519849643111229</v>
+        <v>0.02254565432667732</v>
       </c>
       <c r="G12" t="n">
-        <v>200</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D13" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>98.90%</t>
+          <t>99.41%</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.04548755288124084</v>
+        <v>0.02295735850930214</v>
       </c>
       <c r="G13" t="n">
-        <v>177</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>0.01</v>
       </c>
       <c r="D14" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>98.90%</t>
+          <t>99.41%</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.04569880664348602</v>
+        <v>0.02491552941501141</v>
       </c>
       <c r="G14" t="n">
-        <v>138</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D15" t="n">
         <v>0.01</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>98.90%</t>
+          <t>99.41%</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.05968093872070312</v>
+        <v>0.02533893659710884</v>
       </c>
       <c r="G15" t="n">
-        <v>200</v>
+        <v>169</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -878,20 +878,20 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>98.88%</t>
+          <t>99.40%</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.04489697143435478</v>
+        <v>0.02327304147183895</v>
       </c>
       <c r="G16" t="n">
-        <v>126</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -907,20 +907,20 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>98.88%</t>
+          <t>99.40%</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.04608981311321259</v>
+        <v>0.03213371708989143</v>
       </c>
       <c r="G17" t="n">
-        <v>128</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -936,11 +936,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>98.87%</t>
+          <t>99.40%</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.04566379263997078</v>
+        <v>0.03226776048541069</v>
       </c>
       <c r="G18" t="n">
         <v>200</v>
@@ -949,7 +949,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -965,11 +965,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>98.87%</t>
+          <t>99.40%</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.05665659531950951</v>
+        <v>0.03308005630970001</v>
       </c>
       <c r="G19" t="n">
         <v>200</v>
@@ -978,65 +978,65 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>98.83%</t>
+          <t>99.39%</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.04549912363290787</v>
+        <v>0.02737968228757381</v>
       </c>
       <c r="G20" t="n">
-        <v>31</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D21" t="n">
         <v>0.01</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>98.83%</t>
+          <t>99.39%</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.04722948372364044</v>
+        <v>0.03441743180155754</v>
       </c>
       <c r="G21" t="n">
-        <v>200</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1045,32 +1045,32 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>98.83%</t>
+          <t>99.38%</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.04763741418719292</v>
+        <v>0.0245085135102272</v>
       </c>
       <c r="G22" t="n">
-        <v>16</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1081,40 +1081,40 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>98.83%</t>
+          <t>99.38%</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.04780047014355659</v>
+        <v>0.03291580453515053</v>
       </c>
       <c r="G23" t="n">
-        <v>155</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D24" t="n">
         <v>0.01</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>98.83%</t>
+          <t>99.37%</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.05798466131091118</v>
+        <v>0.02419018372893333</v>
       </c>
       <c r="G24" t="n">
         <v>200</v>
@@ -1123,36 +1123,36 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>98.80%</t>
+          <t>99.37%</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.04652499780058861</v>
+        <v>0.02500960789620876</v>
       </c>
       <c r="G25" t="n">
-        <v>30</v>
+        <v>133</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1168,20 +1168,20 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>98.80%</t>
+          <t>99.36%</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.06030760332942009</v>
+        <v>0.02391756512224674</v>
       </c>
       <c r="G26" t="n">
-        <v>148</v>
+        <v>169</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1190,21 +1190,21 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>98.78%</t>
+          <t>99.36%</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.04723025485873222</v>
+        <v>0.02533596754074097</v>
       </c>
       <c r="G27" t="n">
-        <v>43</v>
+        <v>116</v>
       </c>
     </row>
     <row r="28">
@@ -1215,60 +1215,60 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>0.01</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>98.77%</t>
+          <t>99.36%</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.04300843179225922</v>
+        <v>0.02554901130497456</v>
       </c>
       <c r="G28" t="n">
-        <v>25</v>
+        <v>123</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>0.01</v>
       </c>
       <c r="D29" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>98.77%</t>
+          <t>99.36%</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.06339021027088165</v>
+        <v>0.02582393400371075</v>
       </c>
       <c r="G29" t="n">
-        <v>131</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1284,11 +1284,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>98.75%</t>
+          <t>99.36%</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.04327041655778885</v>
+        <v>0.02729618363082409</v>
       </c>
       <c r="G30" t="n">
         <v>18</v>
@@ -1313,14 +1313,14 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>98.72%</t>
+          <t>99.36%</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.05923495814204216</v>
+        <v>0.03297282010316849</v>
       </c>
       <c r="G31" t="n">
-        <v>200</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32">
@@ -1342,14 +1342,14 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>98.70%</t>
+          <t>99.17%</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0.06183937564492226</v>
+        <v>0.03740376234054565</v>
       </c>
       <c r="G32" t="n">
-        <v>166</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33">
@@ -1371,14 +1371,14 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>98.27%</t>
+          <t>99.15%</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0.0756736621260643</v>
+        <v>0.04128008708357811</v>
       </c>
       <c r="G33" t="n">
-        <v>41</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finito di correggere commenti e nomi in italiano
Sistemato tutti i commenti e messo tutte le variabili ininlgese con commenti in italiano
</commit_message>
<xml_diff>
--- a/export_dati/04_Step4B_Risultati_TensorFlow.xlsx
+++ b/export_dati/04_Step4B_Risultati_TensorFlow.xlsx
@@ -461,14 +461,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -476,16 +476,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.0222802422940731</v>
+        <v>0.02557707205414772</v>
       </c>
       <c r="G2" t="n">
-        <v>19</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -494,32 +494,32 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>99.45%</t>
+          <t>99.44%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.0223421435803175</v>
+        <v>0.02507789060473442</v>
       </c>
       <c r="G3" t="n">
-        <v>10</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -530,14 +530,14 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>99.45%</t>
+          <t>99.42%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.02356160245835781</v>
+        <v>0.02373884245753288</v>
       </c>
       <c r="G4" t="n">
-        <v>56</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
@@ -548,31 +548,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D5" t="n">
         <v>0.0001</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>99.45%</t>
+          <t>99.42%</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.02463765628635883</v>
+        <v>0.02523415349423885</v>
       </c>
       <c r="G5" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -581,27 +581,27 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D6" t="n">
         <v>0.0001</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>99.43%</t>
+          <t>99.42%</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.0230771079659462</v>
+        <v>0.0231925155967474</v>
       </c>
       <c r="G6" t="n">
-        <v>12</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -613,18 +613,18 @@
         <v>0.005</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>99.43%</t>
+          <t>99.42%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.02559859491884708</v>
+        <v>0.02568869851529598</v>
       </c>
       <c r="G7" t="n">
-        <v>31</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8">
@@ -646,14 +646,14 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>99.42%</t>
+          <t>99.41%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.02207266725599766</v>
+        <v>0.02353743277490139</v>
       </c>
       <c r="G8" t="n">
-        <v>21</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9">
@@ -675,20 +675,20 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>99.42%</t>
+          <t>99.41%</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.02410629577934742</v>
+        <v>0.02487782202661037</v>
       </c>
       <c r="G9" t="n">
-        <v>38</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -697,21 +697,21 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>99.42%</t>
+          <t>99.41%</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.0244292039424181</v>
+        <v>0.02550549060106277</v>
       </c>
       <c r="G10" t="n">
-        <v>42</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11">
@@ -722,7 +722,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -733,14 +733,14 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>99.42%</t>
+          <t>99.40%</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.0225406214594841</v>
+        <v>0.02387422136962414</v>
       </c>
       <c r="G11" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
@@ -762,20 +762,20 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>99.42%</t>
+          <t>99.39%</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.02254565432667732</v>
+        <v>0.02249640226364136</v>
       </c>
       <c r="G12" t="n">
-        <v>38</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -784,21 +784,21 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D13" t="n">
         <v>0.0001</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>99.41%</t>
+          <t>99.39%</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.02295735850930214</v>
+        <v>0.02437690272927284</v>
       </c>
       <c r="G13" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
@@ -813,27 +813,27 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D14" t="n">
         <v>0.0001</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>99.41%</t>
+          <t>99.39%</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.02491552941501141</v>
+        <v>0.02534238621592522</v>
       </c>
       <c r="G14" t="n">
-        <v>31</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -842,56 +842,56 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>99.41%</t>
+          <t>99.38%</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.02533893659710884</v>
+        <v>0.02457114681601524</v>
       </c>
       <c r="G15" t="n">
-        <v>169</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D16" t="n">
         <v>0.0001</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>99.40%</t>
+          <t>99.38%</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.02327304147183895</v>
+        <v>0.02510046400129795</v>
       </c>
       <c r="G16" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -903,18 +903,18 @@
         <v>0.01</v>
       </c>
       <c r="D17" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>99.40%</t>
+          <t>99.37%</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.03213371708989143</v>
+        <v>0.02499684318900108</v>
       </c>
       <c r="G17" t="n">
-        <v>200</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
@@ -936,11 +936,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>99.40%</t>
+          <t>99.37%</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.03226776048541069</v>
+        <v>0.03411969169974327</v>
       </c>
       <c r="G18" t="n">
         <v>200</v>
@@ -949,59 +949,59 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D19" t="n">
         <v>0.01</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>99.40%</t>
+          <t>99.37%</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.03308005630970001</v>
+        <v>0.02635023184120655</v>
       </c>
       <c r="G19" t="n">
-        <v>200</v>
+        <v>187</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C20" t="n">
         <v>0.01</v>
       </c>
       <c r="D20" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>99.39%</t>
+          <t>99.37%</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.02737968228757381</v>
+        <v>0.0277490820735693</v>
       </c>
       <c r="G20" t="n">
-        <v>63</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21">
@@ -1016,27 +1016,27 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D21" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>99.39%</t>
+          <t>99.36%</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.03441743180155754</v>
+        <v>0.0250148568302393</v>
       </c>
       <c r="G21" t="n">
-        <v>117</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1045,21 +1045,21 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D22" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>99.38%</t>
+          <t>99.36%</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.0245085135102272</v>
+        <v>0.02641059458255768</v>
       </c>
       <c r="G22" t="n">
-        <v>143</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23">
@@ -1074,47 +1074,47 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D23" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>99.38%</t>
+          <t>99.34%</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.03291580453515053</v>
+        <v>0.02658053115010262</v>
       </c>
       <c r="G23" t="n">
-        <v>115</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D24" t="n">
         <v>0.01</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>99.37%</t>
+          <t>99.34%</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.02419018372893333</v>
+        <v>0.03236968815326691</v>
       </c>
       <c r="G24" t="n">
         <v>200</v>
@@ -1132,61 +1132,61 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D25" t="n">
         <v>0.01</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>99.37%</t>
+          <t>99.33%</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.02500960789620876</v>
+        <v>0.02814244292676449</v>
       </c>
       <c r="G25" t="n">
-        <v>133</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D26" t="n">
         <v>0.01</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>99.36%</t>
+          <t>99.33%</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.02391756512224674</v>
+        <v>0.03730258345603943</v>
       </c>
       <c r="G26" t="n">
-        <v>169</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1197,14 +1197,14 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>99.36%</t>
+          <t>99.30%</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.02533596754074097</v>
+        <v>0.03023265302181244</v>
       </c>
       <c r="G27" t="n">
-        <v>116</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28">
@@ -1226,20 +1226,20 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>99.36%</t>
+          <t>99.29%</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.02554901130497456</v>
+        <v>0.03068902343511581</v>
       </c>
       <c r="G28" t="n">
-        <v>123</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1251,18 +1251,18 @@
         <v>0.01</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>99.36%</t>
+          <t>99.29%</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.02582393400371075</v>
+        <v>0.03561601415276527</v>
       </c>
       <c r="G29" t="n">
-        <v>24</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30">
@@ -1273,25 +1273,25 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>99.36%</t>
+          <t>99.29%</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.02729618363082409</v>
+        <v>0.03779834136366844</v>
       </c>
       <c r="G30" t="n">
-        <v>18</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1313,14 +1313,14 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>99.36%</t>
+          <t>99.27%</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.03297282010316849</v>
+        <v>0.03537554293870926</v>
       </c>
       <c r="G31" t="n">
-        <v>142</v>
+        <v>200</v>
       </c>
     </row>
     <row r="32">
@@ -1335,21 +1335,21 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D32" t="n">
         <v>0.01</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>99.17%</t>
+          <t>99.27%</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0.03740376234054565</v>
+        <v>0.03618545085191727</v>
       </c>
       <c r="G32" t="n">
-        <v>73</v>
+        <v>160</v>
       </c>
     </row>
     <row r="33">
@@ -1371,14 +1371,14 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>99.15%</t>
+          <t>99.19%</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0.04128008708357811</v>
+        <v>0.05016370117664337</v>
       </c>
       <c r="G33" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ultime correzioni per stesura tesi
Sistemato alcune piccole imprecisioni e rigenerato esito in modo da poter incollarlo nella tesi
</commit_message>
<xml_diff>
--- a/export_dati/04_Step4B_Risultati_TensorFlow.xlsx
+++ b/export_dati/04_Step4B_Risultati_TensorFlow.xlsx
@@ -465,27 +465,27 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D2" t="n">
         <v>0.0001</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>99.54%</t>
+          <t>99.55%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.02023756131529808</v>
+        <v>0.02090154588222504</v>
       </c>
       <c r="G2" t="n">
-        <v>33</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -505,10 +505,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.02042479626834393</v>
+        <v>0.0205504521727562</v>
       </c>
       <c r="G3" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -519,7 +519,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -534,21 +534,21 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.02070550620555878</v>
+        <v>0.01985298283398151</v>
       </c>
       <c r="G4" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -563,16 +563,16 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.01982523314654827</v>
+        <v>0.0203405674546957</v>
       </c>
       <c r="G5" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -588,25 +588,25 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>99.51%</t>
+          <t>99.52%</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.01979403384029865</v>
+        <v>0.02095773629844189</v>
       </c>
       <c r="G6" t="n">
-        <v>40</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -617,20 +617,20 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>99.51%</t>
+          <t>99.52%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.02014796622097492</v>
+        <v>0.02029022760689259</v>
       </c>
       <c r="G7" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -642,24 +642,24 @@
         <v>0.005</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>99.51%</t>
+          <t>99.52%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.02175948396325111</v>
+        <v>0.02077257819473743</v>
       </c>
       <c r="G8" t="n">
-        <v>189</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -668,56 +668,56 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D9" t="n">
         <v>0.0001</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>99.50%</t>
+          <t>99.51%</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.02001300640404224</v>
+        <v>0.02118460834026337</v>
       </c>
       <c r="G9" t="n">
-        <v>15</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>0.005</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>99.50%</t>
+          <t>99.51%</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.02089585550129414</v>
+        <v>0.02162229642271996</v>
       </c>
       <c r="G10" t="n">
-        <v>105</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -733,20 +733,20 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>99.50%</t>
+          <t>99.51%</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.02170435152947903</v>
+        <v>0.02171079255640507</v>
       </c>
       <c r="G11" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -762,43 +762,43 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>99.49%</t>
+          <t>99.50%</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.0211963877081871</v>
+        <v>0.01976898498833179</v>
       </c>
       <c r="G12" t="n">
-        <v>99</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>(32,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D13" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>99.48%</t>
+          <t>99.50%</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.02159576490521431</v>
+        <v>0.02167397551238537</v>
       </c>
       <c r="G13" t="n">
-        <v>200</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14">
@@ -820,20 +820,20 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>99.48%</t>
+          <t>99.49%</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.0226092841476202</v>
+        <v>0.02214518934488297</v>
       </c>
       <c r="G14" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -842,10 +842,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -853,16 +853,16 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.02159471809864044</v>
+        <v>0.02175879664719105</v>
       </c>
       <c r="G15" t="n">
-        <v>186</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -874,7 +874,7 @@
         <v>0.005</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -882,10 +882,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.0226493813097477</v>
+        <v>0.02270972914993763</v>
       </c>
       <c r="G16" t="n">
-        <v>39</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17">
@@ -907,14 +907,14 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>99.47%</t>
+          <t>99.48%</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.0204023327678442</v>
+        <v>0.0205727219581604</v>
       </c>
       <c r="G17" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18">
@@ -936,11 +936,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>99.47%</t>
+          <t>99.48%</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.02136849239468575</v>
+        <v>0.02129850722849369</v>
       </c>
       <c r="G18" t="n">
         <v>200</v>
@@ -949,30 +949,30 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D19" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>99.47%</t>
+          <t>99.48%</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.02168705314397812</v>
+        <v>0.02321567572653294</v>
       </c>
       <c r="G19" t="n">
-        <v>200</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20">
@@ -983,7 +983,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -998,10 +998,10 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.02214073017239571</v>
+        <v>0.02178866229951382</v>
       </c>
       <c r="G20" t="n">
-        <v>121</v>
+        <v>200</v>
       </c>
     </row>
     <row r="21">
@@ -1012,36 +1012,36 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D21" t="n">
         <v>0.01</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>99.47%</t>
+          <t>99.46%</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.02262848243117332</v>
+        <v>0.02169731073081493</v>
       </c>
       <c r="G21" t="n">
-        <v>106</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1052,20 +1052,20 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>99.45%</t>
+          <t>99.46%</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.02172020636498928</v>
+        <v>0.02316782809793949</v>
       </c>
       <c r="G22" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32,)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1077,24 +1077,24 @@
         <v>0.01</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>99.45%</t>
+          <t>99.44%</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.02382347919046879</v>
+        <v>0.02283337898552418</v>
       </c>
       <c r="G23" t="n">
-        <v>28</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1114,45 +1114,45 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.02955211140215397</v>
+        <v>0.02317501045763493</v>
       </c>
       <c r="G24" t="n">
-        <v>200</v>
+        <v>98</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C25" t="n">
         <v>0.01</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>99.43%</t>
+          <t>99.44%</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.02326660975813866</v>
+        <v>0.0313618928194046</v>
       </c>
       <c r="G25" t="n">
-        <v>18</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1168,11 +1168,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>99.43%</t>
+          <t>99.41%</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.03086062148213387</v>
+        <v>0.03196803480386734</v>
       </c>
       <c r="G26" t="n">
         <v>200</v>
@@ -1197,43 +1197,43 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>99.42%</t>
+          <t>99.40%</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.02996851690113544</v>
+        <v>0.03058201260864735</v>
       </c>
       <c r="G27" t="n">
-        <v>143</v>
+        <v>121</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>(64,)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="D28" t="n">
         <v>0.01</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>99.42%</t>
+          <t>99.40%</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.02358184009790421</v>
+        <v>0.03107140399515629</v>
       </c>
       <c r="G28" t="n">
-        <v>122</v>
+        <v>200</v>
       </c>
     </row>
     <row r="29">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1255,25 +1255,25 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>99.42%</t>
+          <t>99.39%</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.03033427149057388</v>
+        <v>0.02945279516279697</v>
       </c>
       <c r="G29" t="n">
-        <v>200</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(32, 16)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>relu</t>
+          <t>tanh</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1284,20 +1284,20 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>99.42%</t>
+          <t>99.39%</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.0346190445125103</v>
+        <v>0.03123926371335983</v>
       </c>
       <c r="G30" t="n">
-        <v>66</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1306,32 +1306,32 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D31" t="n">
         <v>0.01</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>99.41%</t>
+          <t>99.39%</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.02977978810667992</v>
+        <v>0.03591442108154297</v>
       </c>
       <c r="G31" t="n">
-        <v>193</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>(32, 16)</t>
+          <t>(64, 32)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>tanh</t>
+          <t>relu</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1346,16 +1346,16 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0.03307312354445457</v>
+        <v>0.03633152693510056</v>
       </c>
       <c r="G32" t="n">
-        <v>73</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>(64, 32)</t>
+          <t>(64,)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1371,14 +1371,14 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>99.39%</t>
+          <t>99.38%</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0.03900574892759323</v>
+        <v>0.02633390389382839</v>
       </c>
       <c r="G33" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>